<commit_message>
map the known legacy metamorphic and sedimentary leaves to the material tree
A MATERIAL_SPECIALS table keys each rooted legacy slug to the path the
geologist's mapping instructions assign it (Gneiss and friends sit under
strongly_metamorphosed, Carbonate/Ironstone under the biochemical branch,
SiliceousBiogenic and MixedCarb-Siliciclastic are hybrid rocks...). The values
their table marks 'record to review' (MechanicallyBroken, Meta-Carbonate,
Meta-Ultramafic) are deliberately absent so those rows keep skipping into the
import log. The spreadsheet mirrors the mappings on a new 'Material remaps'
tab.
</commit_message>
<xml_diff>
--- a/docs/legacy-import-mapping.xlsx
+++ b/docs/legacy-import-mapping.xlsx
@@ -7,6 +7,7 @@
     <sheet name="1-x mapping" sheetId="3" r:id="rId3"/>
     <sheet name="Unmapped columns" sheetId="4" r:id="rId4"/>
     <sheet name="Unknown values" sheetId="5" r:id="rId5"/>
+    <sheet name="Material remaps" sheetId="6" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -518,12 +519,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">classification slugged to a dot path (rock families prefixed 'rock.'), kept to its longest valid prefix; the coarse material root is used only when there is no classification</t>
+          <t xml:space="preserve">classification slugged to a dot path (rock families prefixed 'rock.'), remapped by the MATERIAL_SPECIALS table (import script) when the legacy leaf sits elsewhere in the new tree, kept to its longest valid prefix; the coarse material root is used only when there is no classification</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A path the material tree does not support skips the row (~7,700). We never truncate to a coarser path, and never fall back to the material root when a classification exists.</t>
+          <t xml:space="preserve">A path the material tree does not support skips the row. We never truncate to a coarser path, and never fall back to the material root when a classification exists; the MATERIAL_SPECIALS targets follow the geologist's instructions (see the 'Material remaps' tab), which leave MechanicallyBroken / Meta-Carbonate / Meta-Ultramafic to review (still skipped).</t>
         </is>
       </c>
     </row>
@@ -1453,27 +1454,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Calc-Silicate</t>
+          <t xml:space="preserve">Metamorphic&gt;MechanicallyBroken</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.calc_silicate</t>
+          <t xml:space="preserve">rock.metamorphic.mechanically_broken</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic has only weakly_metamorphosed / strongly_metamorphosed as children, and the new term carries a '_rock' suffix.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.calc_silicate_rock</t>
+          <t xml:space="preserve">No mechanically-broken / fault-rock branch in the new tree; it only lists individual leaves (mylonite, impactite).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Marked 'record to review' in the expert mapping table; decide the target path, then map it in the import script.</t>
         </is>
       </c>
     </row>
@@ -1485,27 +1481,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Gneiss</t>
+          <t xml:space="preserve">Metamorphic&gt;Meta-Carbonate</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.gneiss</t>
+          <t xml:space="preserve">rock.metamorphic.meta_carbonate</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position.</t>
+          <t xml:space="preserve">Absent under that name: metamorphosed sediments hang under weakly_metamorphosed.meta_sedimentary_rock.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.gneiss</t>
+          <t xml:space="preserve">rock.metamorphic.weakly_metamorphosed.meta_sedimentary_rock.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Marked 'record to review' in the expert mapping table; decide the target path, then map it in the import script.</t>
         </is>
       </c>
     </row>
@@ -1517,22 +1513,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Granofels</t>
+          <t xml:space="preserve">Metamorphic&gt;Meta-Ultramafic</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.granofels</t>
+          <t xml:space="preserve">rock.metamorphic.meta_ultramafic</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The term is absent from the material tree at any depth.</t>
+          <t xml:space="preserve">Absent: 'ultramafic' exists only as an igneous branch, with no metamorphosed counterpart.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.igneous.plutonic.ultramafic (not equivalent, it is not metamorphic)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add the term to the material tree first, then map it.</t>
+          <t xml:space="preserve">Marked 'record to review' in the expert mapping table; decide the target path, then map it in the import script.</t>
         </is>
       </c>
     </row>
@@ -1544,27 +1545,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Granulite</t>
+          <t xml:space="preserve">Ore&gt;Sulfide</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.granulite</t>
+          <t xml:space="preserve">ore.sulfide</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position.</t>
+          <t xml:space="preserve">'Ore' is neither a rock family (so no 'rock.' prefix is applied) nor a material root, so the path has no known root.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.granulite (also felsic_granulite / mafic_granulite)</t>
+          <t xml:space="preserve">rock.hydrothermal.sulfide</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. Ore itself stays a genetic qualifier the tree does not carry.</t>
         </is>
       </c>
     </row>
@@ -1576,22 +1577,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;MechanicallyBroken</t>
+          <t xml:space="preserve">Other</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.mechanically_broken</t>
+          <t xml:space="preserve">other</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No mechanically-broken / fault-rock branch in the new tree; it only lists individual leaves (mylonite, impactite).</t>
+          <t xml:space="preserve">material_id root with no counterpart: the new roots are rock, sediment, mineral, fossil, synthetic_rock_mineral, extraterrestrial_rock.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add the term to the material tree first, then map it.</t>
+          <t xml:space="preserve">Needs a new field or vocabulary in the domain, not just a mapping.</t>
         </is>
       </c>
     </row>
@@ -1603,27 +1604,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Meta-Carbonate</t>
+          <t xml:space="preserve">Soil</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.meta_carbonate</t>
+          <t xml:space="preserve">soil</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Absent under that name: metamorphosed sediments hang under weakly_metamorphosed.meta_sedimentary_rock.</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.metamorphic.weakly_metamorphosed.meta_sedimentary_rock.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
+          <t xml:space="preserve">material_id root with no counterpart: the new roots are rock, sediment, mineral, fossil, synthetic_rock_mineral, extraterrestrial_rock.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Needs a new field or vocabulary in the domain, not just a mapping.</t>
         </is>
       </c>
     </row>
@@ -1635,27 +1631,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Meta-Ultramafic</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.meta_ultramafic</t>
+          <t xml:space="preserve">xenolithic.igneous.plutonic</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Absent: 'ultramafic' exists only as an igneous branch, with no metamorphosed counterpart.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.igneous.plutonic.ultramafic (not equivalent, it is not metamorphic)</t>
+          <t xml:space="preserve">rock.igneous.plutonic</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add the term to the material tree first, then map it.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1667,27 +1663,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Schist</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Felsic</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.schist</t>
+          <t xml:space="preserve">xenolithic.igneous.plutonic.felsic</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.schist (also mica_schist / greenschist)</t>
+          <t xml:space="preserve">rock.igneous.plutonic.felsic</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1699,27 +1695,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metamorphic&gt;Slate</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Intermediate</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.slate</t>
+          <t xml:space="preserve">xenolithic.igneous.plutonic.intermediate</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.slate</t>
+          <t xml:space="preserve">rock.igneous.plutonic.intermediate</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1731,27 +1727,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ore&gt;Sulfide</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Mafic</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ore.sulfide</t>
+          <t xml:space="preserve">xenolithic.igneous.plutonic.mafic</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">'Ore' is neither a rock family (so no 'rock.' prefix is applied) nor a material root, so the path has no known root.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.hydrothermal.sulfide</t>
+          <t xml:space="preserve">rock.igneous.plutonic.mafic</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. Ore itself stays a genetic qualifier the tree does not carry.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1763,22 +1759,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Ultramafic</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">other</t>
+          <t xml:space="preserve">xenolithic.igneous.plutonic.ultramafic</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">material_id root with no counterpart: the new roots are rock, sediment, mineral, fossil, synthetic_rock_mineral, extraterrestrial_rock.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.igneous.plutonic.ultramafic</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs a new field or vocabulary in the domain, not just a mapping.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1791,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;Carbonate</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.carbonate</t>
+          <t xml:space="preserve">xenolithic.igneous.volcanic</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position. The new term also carries a '_rock' suffix.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
+          <t xml:space="preserve">rock.igneous.volcanic</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1822,27 +1823,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;ConglomerateAndOrBreccia</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Felsic</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.conglomerate_and_or_breccia</t>
+          <t xml:space="preserve">xenolithic.igneous.volcanic.felsic</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The combined legacy term has no equivalent; the new tree does not group conglomerate and breccia together.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.clastic_sedimentary_rock.paraconglomerate</t>
+          <t xml:space="preserve">rock.igneous.volcanic.felsic</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ambiguous: the legacy value does not say which of the two it is.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1854,27 +1855,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;Ironstone</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Intermediate</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.ironstone</t>
+          <t xml:space="preserve">xenolithic.igneous.volcanic.intermediate</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.biochemical_and_chemical_sedimentary_rock.ironstone</t>
+          <t xml:space="preserve">rock.igneous.volcanic.intermediate</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1886,27 +1887,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;MixedCarb-Siliciclastic</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Mafic</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.mixed_carb_siliciclastic</t>
+          <t xml:space="preserve">xenolithic.igneous.volcanic.mafic</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Absent under that name: the new tree calls a carbonate / siliciclastic mixture 'hybrid'.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.hybrid_sedimentary_rock</t>
+          <t xml:space="preserve">rock.igneous.volcanic.mafic</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1918,27 +1919,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;SiliceousBiogenic</t>
+          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Ultramafic</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.siliceous_biogenic</t>
+          <t xml:space="preserve">xenolithic.igneous.volcanic.ultramafic</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position. The new term is named siliceous_rock.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.biochemical_and_chemical_sedimentary_rock.siliceous_rock</t>
+          <t xml:space="preserve">rock.igneous.volcanic.ultramafic</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1950,27 +1951,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;Siliciclastic</t>
+          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Gneiss</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.siliciclastic</t>
+          <t xml:space="preserve">xenolithic.metamorphic.gneiss</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position. The new term carries a '_sedimentary_rock' suffix.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. The leaf also sits deeper.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.clastic_sedimentary_rock.siliciclastic_sedimentary_rock</t>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.gneiss</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -1982,27 +1983,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sedimentary&gt;Volcaniclastic</t>
+          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Granulite</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.volcaniclastic</t>
+          <t xml:space="preserve">xenolithic.metamorphic.granulite</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The leaf exists in the new tree but sits deeper, so the legacy path is not a supported segment sequence at that position. The new term carries a '_rock' suffix.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. The leaf also sits deeper.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.sedimentary.volcaniclastic_rock</t>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.granulite</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -2014,22 +2015,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Soil</t>
+          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Meta-Carbonate</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">soil</t>
+          <t xml:space="preserve">xenolithic.metamorphic.meta_carbonate</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">material_id root with no counterpart: the new roots are rock, sediment, mineral, fossil, synthetic_rock_mineral, extraterrestrial_rock.</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. 'meta_carbonate' is also absent under that name.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.weakly_metamorphosed.meta_sedimentary_rock.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs a new field or vocabulary in the domain, not just a mapping.</t>
+          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
         </is>
       </c>
     </row>
@@ -2041,527 +2047,111 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic</t>
+          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Meta-Ultramafic</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">xenolithic.igneous.plutonic</t>
+          <t xml:space="preserve">xenolithic.metamorphic.meta_ultramafic</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.plutonic</t>
+          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. 'meta_ultramafic' is also absent from the tree.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
+          <t xml:space="preserve">Add the term to the material tree first, then map it.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">resource_type</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Felsic</t>
+          <t xml:space="preserve">Grab</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">xenolithic.igneous.plutonic.felsic</t>
+          <t xml:space="preserve">grab</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
+          <t xml:space="preserve">Neither a nature nor a node in the sample-type tree (roots: core, dredge, individual_sample, serie_of_sample, inapplicable).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.igneous.plutonic.felsic</t>
+          <t xml:space="preserve">collection method 'grab' rather than a type</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
+          <t xml:space="preserve">Decide whether a legacy grab feeds collection_method instead of type.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">resource_type</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Intermediate</t>
+          <t xml:space="preserve">Outcrop</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">xenolithic.igneous.plutonic.intermediate</t>
+          <t xml:space="preserve">outcrop</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
+          <t xml:space="preserve">Not a nature, and the type tree has no outcrop node.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rock.igneous.plutonic.intermediate</t>
+          <t xml:space="preserve">core.outcrop_preserved_stratigraphy (a core attribute, not an outcrop sample)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
+          <t xml:space="preserve">Needs a type-tree decision: an outcrop sample is not a core.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">resource_type</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Mafic</t>
+          <t xml:space="preserve">Site</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">xenolithic.igneous.plutonic.mafic</t>
+          <t xml:space="preserve">site</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.plutonic.mafic</t>
+          <t xml:space="preserve">A site is a place, not a physical form or a sampling taxonomy: no nature and no type node.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Plutonic&gt;Ultramafic</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.plutonic.ultramafic</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.plutonic.ultramafic</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.volcanic</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.volcanic</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Felsic</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.volcanic.felsic</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.volcanic.felsic</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Intermediate</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.volcanic.intermediate</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.volcanic.intermediate</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Mafic</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.volcanic.mafic</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.volcanic.mafic</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Igneous&gt;Volcanic&gt;Ultramafic</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.igneous.volcanic.ultramafic</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path.</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.igneous.volcanic.ultramafic</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Gneiss</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.metamorphic.gneiss</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. The leaf also sits deeper.</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.gneiss</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Granulite</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.metamorphic.granulite</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. The leaf also sits deeper.</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.granulite</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Meta-Carbonate</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.metamorphic.meta_carbonate</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. 'meta_carbonate' is also absent under that name.</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rock.metamorphic.weakly_metamorphosed.meta_sedimentary_rock.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Map the legacy label in the import script: the target path exists. The xenolith qualifier is lost either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic&gt;Metamorphic&gt;Meta-Ultramafic</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">xenolithic.metamorphic.meta_ultramafic</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xenolithic is not a rock family, so the 'rock.' prefix is not applied and the path has no root the tree knows; there is no xenolith root or qualifier in the new model, only the underlying rock path. 'meta_ultramafic' is also absent from the tree.</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add the term to the material tree first, then map it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">resource_type</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grab</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grab</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Neither a nature nor a node in the sample-type tree (roots: core, dredge, individual_sample, serie_of_sample, inapplicable).</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">collection method 'grab' rather than a type</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decide whether a legacy grab feeds collection_method instead of type.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">resource_type</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outcrop</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">outcrop</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not a nature, and the type tree has no outcrop node.</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core.outcrop_preserved_stratigraphy (a core attribute, not an outcrop sample)</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Needs a type-tree decision: an outcrop sample is not a core.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">resource_type</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Site</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">site</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A site is a place, not a physical form or a sampling taxonomy: no nature and no type node.</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Out of scope: the new model has no site-level record.</t>
         </is>
@@ -2570,4 +2160,194 @@
   </sheetData>
   <autoFilter ref="A1:F43"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legacy value</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imported material path</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Calc-Silicate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.calc_silicate_rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Gneiss</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.gneiss</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Granofels</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.granofels</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">granofels was added to the material tree for this mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Granulite</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.granulite</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Schist</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.schist</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metamorphic&gt;Slate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.metamorphic.strongly_metamorphosed.slate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;Carbonate</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.biochemical_and_chemical_sedimentary_rock.carbonate_rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;ConglomerateAndOrBreccia</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.clastic_sedimentary_rock.paraconglomerate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;Ironstone</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.biochemical_and_chemical_sedimentary_rock.ironstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;MixedCarb-Siliciclastic</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.hybrid_sedimentary_rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;SiliceousBiogenic</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.hybrid_sedimentary_rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;Siliciclastic</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.clastic_sedimentary_rock.siliciclastic_sedimentary_rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sedimentary&gt;Volcaniclastic</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rock.sedimentary.volcaniclastic_rock</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>